<commit_message>
Actualizacao grafico do Grants
</commit_message>
<xml_diff>
--- a/Qualidade_Sessoes.xlsx
+++ b/Qualidade_Sessoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -424,17 +424,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>26-Feb-2026</t>
+          <t>16-Apr-2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3918786000010039074</t>
+          <t>3918786000010055064</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -471,7 +471,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -481,17 +481,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -501,17 +501,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>05-Mar-2026</t>
+          <t>14-Apr-2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3918786000010039072</t>
+          <t>3918786000010050002</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -528,7 +528,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -558,17 +558,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>19-Feb-2026</t>
+          <t>26-Feb-2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3918786000010039070</t>
+          <t>3918786000010039074</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -615,17 +615,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>14-Feb-2026</t>
+          <t>05-Mar-2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3918786000010039068</t>
+          <t>3918786000010039072</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -642,7 +642,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -652,12 +652,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -672,17 +672,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>25-Mar-2026</t>
+          <t>19-Feb-2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3918786000010039066</t>
+          <t>3918786000010039070</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -699,47 +699,47 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MUELEGE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>14-Feb-2026</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TOPELANE</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Sessão_2</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>18-Apr-2026</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3918786000010039064</t>
+          <t>3918786000010039068</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -756,7 +756,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -786,17 +786,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>13-Feb-2026</t>
+          <t>25-Mar-2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3918786000010039062</t>
+          <t>3918786000010039066</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -813,7 +813,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>04-Mar-2026</t>
+          <t>18-Apr-2026</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3918786000010039060</t>
+          <t>3918786000010039064</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -870,7 +870,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -900,17 +900,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>04-Mar-2026</t>
+          <t>13-Feb-2026</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3918786000010039058</t>
+          <t>3918786000010039062</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>25-Feb-2026</t>
+          <t>04-Mar-2026</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>3918786000010039056</t>
+          <t>3918786000010039060</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>18-Feb-2026</t>
+          <t>04-Mar-2026</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3918786000010039054</t>
+          <t>3918786000010039058</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1071,17 +1071,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>13-Feb-2026</t>
+          <t>25-Feb-2026</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3918786000010039052</t>
+          <t>3918786000010039056</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1108,12 +1108,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sessão_9</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1128,17 +1128,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>14-Apr-2026</t>
+          <t>18-Feb-2026</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>3918786000010039050</t>
+          <t>3918786000010039054</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1165,17 +1165,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sessão_8</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10-Apr-2026</t>
+          <t>13-Feb-2026</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3918786000010023384</t>
+          <t>3918786000010039052</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1212,7 +1212,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_9</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1242,17 +1242,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>11-Feb-2026</t>
+          <t>14-Apr-2026</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>3918786000010023382</t>
+          <t>3918786000010039050</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sessão_9</t>
+          <t>Sessão_10</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1299,17 +1299,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08-Apr-2026</t>
+          <t>15-Apr-2026</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>3918786000010023380</t>
+          <t>3918786000010037472</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1326,7 +1326,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1336,12 +1336,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_9</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1356,17 +1356,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13-Feb-2026</t>
+          <t>14-Apr-2026</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3918786000010023378</t>
+          <t>3918786000010037470</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1383,7 +1383,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sessão_7</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>09-Apr-2026</t>
+          <t>10-Apr-2026</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>3918786000010020060</t>
+          <t>3918786000010023384</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1440,7 +1440,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1450,17 +1450,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sessão_9</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1470,17 +1470,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>09-Apr-2026</t>
+          <t>11-Feb-2026</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>3918786000010019064</t>
+          <t>3918786000010023382</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1497,52 +1497,52 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MATHAPUE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sessão_8</t>
+          <t>Sessão_9</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FERNANDES LIMA &amp; TAIRAHA ESQUADRO</t>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>31-Mar-2026</t>
+          <t>08-Apr-2026</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>3918786000010015292</t>
+          <t>3918786000010023380</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Nacala Porto</t>
+          <t>Monapo</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1554,52 +1554,52 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MATHAPUE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sessão_7</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FERNANDES LIMA &amp; TAIRAHA ESQUADRO</t>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>31-Mar-2026</t>
+          <t>13-Feb-2026</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>3918786000010015290</t>
+          <t>3918786000010023378</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Nacala Porto</t>
+          <t>Monapo</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1611,37 +1611,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MATHAPUE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_7</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FERNANDES LIMA &amp; TAIRAHA ESQUADRO</t>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>31-Mar-2026</t>
+          <t>09-Apr-2026</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1651,12 +1651,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>3918786000010015288</t>
+          <t>3918786000010020060</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Nacala Porto</t>
+          <t>Monapo</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1668,52 +1668,52 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MATHAPUE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_9</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FERNANDES LIMA &amp; TAIRAHA ESQUADRO</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>31-Mar-2026</t>
+          <t>09-Apr-2026</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>3918786000010015286</t>
+          <t>3918786000010019064</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Nacala Porto</t>
+          <t>Monapo</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1760,12 +1760,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>3918786000010015284</t>
+          <t>3918786000010015292</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1782,7 +1782,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_7</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1817,12 +1817,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>3918786000010015282</t>
+          <t>3918786000010015290</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1839,7 +1839,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1874,12 +1874,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>3918786000010015280</t>
+          <t>3918786000010015288</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1896,12 +1896,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1931,12 +1931,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>3918786000010015278</t>
+          <t>3918786000010015286</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1953,52 +1953,52 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MATHAPUE</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sessão_9</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
+          <t>FERNANDES LIMA &amp; TAIRAHA ESQUADRO</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08-Apr-2026</t>
+          <t>31-Mar-2026</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>3918786000010011002</t>
+          <t>3918786000010015284</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Nacala Porto</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2010,52 +2010,52 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MATHAPUE</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Sessão_8</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>FERNANDES LIMA &amp; TAIRAHA ESQUADRO</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08-Apr-2026</t>
+          <t>31-Mar-2026</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>3918786000010007188</t>
+          <t>3918786000010015282</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Nacala Porto</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2067,37 +2067,37 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>MATHAPUE</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sessão_8</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>FERNANDES LIMA &amp; TAIRAHA ESQUADRO</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>09-Apr-2026</t>
+          <t>31-Mar-2026</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>3918786000010007186</t>
+          <t>3918786000010015280</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Nacala Porto</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2124,52 +2124,52 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MATHAPUE</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Sessão_9</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>FERNANDES LIMA &amp; TAIRAHA ESQUADRO</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10-Apr-2026</t>
+          <t>31-Mar-2026</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>3918786000010005495</t>
+          <t>3918786000010015278</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Nacala Porto</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2191,17 +2191,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Sessão_7</t>
+          <t>Sessão_9</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2211,17 +2211,17 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>27-Mar-2026</t>
+          <t>08-Apr-2026</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>3918786000009978061</t>
+          <t>3918786000010011002</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2238,7 +2238,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Sessão_7</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2268,17 +2268,17 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>25-Mar-2026</t>
+          <t>08-Apr-2026</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>3918786000009978059</t>
+          <t>3918786000010007188</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2295,7 +2295,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2325,17 +2325,17 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>25-Mar-2026</t>
+          <t>09-Apr-2026</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>3918786000009978057</t>
+          <t>3918786000010007186</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_9</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2382,17 +2382,17 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>11-Mar-2026</t>
+          <t>10-Apr-2026</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>3918786000009978055</t>
+          <t>3918786000010005495</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2409,7 +2409,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_7</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2439,17 +2439,17 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>11-Mar-2026</t>
+          <t>27-Mar-2026</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>3918786000009978053</t>
+          <t>3918786000009978061</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2496,17 +2496,17 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>02-Apr-2026</t>
+          <t>25-Mar-2026</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>3918786000009978051</t>
+          <t>3918786000009978059</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2523,7 +2523,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2533,17 +2533,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Sessão_8</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2553,17 +2553,17 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>02-Apr-2026</t>
+          <t>25-Mar-2026</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>3918786000009975096</t>
+          <t>3918786000009978057</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2580,7 +2580,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2590,17 +2590,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2610,17 +2610,17 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>02-Apr-2026</t>
+          <t>11-Mar-2026</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>3918786000009966138</t>
+          <t>3918786000009978055</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2637,7 +2637,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2652,12 +2652,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Sessão_8</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2667,17 +2667,17 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>01-Apr-2026</t>
+          <t>11-Mar-2026</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>3918786000009966136</t>
+          <t>3918786000009978053</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2694,7 +2694,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2724,17 +2724,17 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>01-Apr-2026</t>
+          <t>02-Apr-2026</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>3918786000009964076</t>
+          <t>3918786000009978051</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2751,7 +2751,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2781,17 +2781,17 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08-Apr-2026</t>
+          <t>02-Apr-2026</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>3918786000009964074</t>
+          <t>3918786000009975096</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2808,7 +2808,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2818,17 +2818,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>01-Apr-2026</t>
+          <t>02-Apr-2026</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>3918786000009964072</t>
+          <t>3918786000009966138</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2865,7 +2865,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2875,17 +2875,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2900,12 +2900,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>3918786000009964070</t>
+          <t>3918786000009966136</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_7</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2957,12 +2957,12 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>3918786000009964068</t>
+          <t>3918786000009964076</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2979,7 +2979,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3009,17 +3009,17 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>01-Apr-2026</t>
+          <t>08-Apr-2026</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>3918786000009964066</t>
+          <t>3918786000009964074</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3036,7 +3036,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3071,12 +3071,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>3918786000009964064</t>
+          <t>3918786000009964072</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -3093,7 +3093,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3103,12 +3103,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Sessão_8</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3123,17 +3123,17 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>31-Mar-2026</t>
+          <t>01-Apr-2026</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>3918786000009964062</t>
+          <t>3918786000009964070</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3150,7 +3150,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3160,17 +3160,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Sessão_8</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3185,12 +3185,12 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>3918786000009962078</t>
+          <t>3918786000009964068</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -3207,7 +3207,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3217,12 +3217,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Sessão_7</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3237,17 +3237,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>24-Mar-2026</t>
+          <t>01-Apr-2026</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>3918786000009962026</t>
+          <t>3918786000009964066</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3264,7 +3264,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3274,12 +3274,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3294,17 +3294,17 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>17-Mar-2026</t>
+          <t>01-Apr-2026</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>3918786000009962024</t>
+          <t>3918786000009964064</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3351,17 +3351,17 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10-Mar-2026</t>
+          <t>31-Mar-2026</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>3918786000009962022</t>
+          <t>3918786000009964062</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3378,7 +3378,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3388,17 +3388,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3408,17 +3408,17 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>03-Mar-2026</t>
+          <t>01-Apr-2026</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>3918786000009962020</t>
+          <t>3918786000009962078</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_7</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>24-Feb-2026</t>
+          <t>24-Mar-2026</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>3918786000009962018</t>
+          <t>3918786000009962026</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3522,17 +3522,17 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>17-Feb-2026</t>
+          <t>17-Mar-2026</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>3918786000009962016</t>
+          <t>3918786000009962024</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3579,17 +3579,17 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>13-Feb-2026</t>
+          <t>10-Mar-2026</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>3918786000009962014</t>
+          <t>3918786000009962022</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3606,7 +3606,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3616,17 +3616,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3636,17 +3636,17 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>26-Mar-2026</t>
+          <t>03-Mar-2026</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>3918786000009891291</t>
+          <t>3918786000009962020</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3663,7 +3663,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3673,17 +3673,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Sessão_7</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3693,17 +3693,17 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>25-Mar-2026</t>
+          <t>24-Feb-2026</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>3918786000009891287</t>
+          <t>3918786000009962018</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3720,7 +3720,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3730,17 +3730,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3750,17 +3750,17 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>25-Mar-2026</t>
+          <t>17-Feb-2026</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>3918786000009888175</t>
+          <t>3918786000009962016</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3777,7 +3777,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3787,17 +3787,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>SERGIO FAUSTO &amp; ZITO JOSIAS</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3807,17 +3807,17 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>19-Mar-2026</t>
+          <t>13-Feb-2026</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>3918786000009886133</t>
+          <t>3918786000009962014</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3834,7 +3834,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3864,17 +3864,17 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>12-Mar-2026</t>
+          <t>26-Mar-2026</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>3918786000009886129</t>
+          <t>3918786000009891291</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3891,7 +3891,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_7</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3921,17 +3921,17 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>18-Feb-2026</t>
+          <t>25-Mar-2026</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>3918786000009856153</t>
+          <t>3918786000009891287</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3948,7 +3948,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3963,12 +3963,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3978,17 +3978,17 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>25-Feb-2026</t>
+          <t>25-Mar-2026</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>3918786000009856149</t>
+          <t>3918786000009888175</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -4005,7 +4005,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4015,17 +4015,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4035,17 +4035,17 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>04-Mar-2026</t>
+          <t>19-Mar-2026</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>3918786000009856145</t>
+          <t>3918786000009886133</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -4072,17 +4072,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+          <t>PAULO ALEXANDRE &amp; TOMAS NHAMPA</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -4092,17 +4092,17 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>19-Feb-2026</t>
+          <t>12-Mar-2026</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>3918786000009856141</t>
+          <t>3918786000009886129</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -4119,7 +4119,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4129,12 +4129,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -4149,17 +4149,17 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>26-Feb-2026</t>
+          <t>18-Feb-2026</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>3918786000009856137</t>
+          <t>3918786000009856153</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -4176,7 +4176,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -4206,17 +4206,17 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>11-Mar-2026</t>
+          <t>25-Feb-2026</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>3918786000009856133</t>
+          <t>3918786000009856149</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -4233,7 +4233,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -4263,17 +4263,17 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>17-Mar-2026</t>
+          <t>04-Mar-2026</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>3918786000009856129</t>
+          <t>3918786000009856145</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -4290,55 +4290,283 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>19-Feb-2026</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>3918786000009856141</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>26-Feb-2026</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>3918786000009856137</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Sessão_5</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>11-Mar-2026</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>3918786000009856133</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Sessão_6</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>17-Mar-2026</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>3918786000009856129</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
         <is>
           <t>RAMIANE</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>Sessão_4</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
         <is>
           <t>19-Mar-2026</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="H74" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t>3918786000009856125</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>Monapo</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -4605,13 +4833,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95F58293-6994-4974-8E2D-DD663C674542}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68735154-487A-4E1C-87E9-E4FEDA786EA4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B00EB8E-3B6B-4087-88E0-334D42B4ED95}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12B360E7-B2FF-4F5F-9D7A-718BD43FB1E1}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69C8AC43-6896-4294-85CB-51E8DF774B78}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F096A08E-736E-49C4-AF82-A89D0D24FF96}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao da pagina de mentoria
</commit_message>
<xml_diff>
--- a/Qualidade_Sessoes.xlsx
+++ b/Qualidade_Sessoes.xlsx
@@ -9876,4 +9876,271 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
+    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B4200DC-FCE5-4054-A69F-C214589C833C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A7E49F4-0F06-4A31-B05F-84A8235AF667}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6891425A-5736-4BB5-AC64-DEB39513C3E9}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao das ultimas sessoes de PI
</commit_message>
<xml_diff>
--- a/Qualidade_Sessoes.xlsx
+++ b/Qualidade_Sessoes.xlsx
@@ -10047,271 +10047,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
-    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DF66064-9E6D-454B-A278-049E0AF7A007}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46159C7B-FEBD-4BA3-BF4F-D67258D0263C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFF3CEA8-968B-4FB1-8983-6A4839D8E81C}"/>
 </file>
</xml_diff>

<commit_message>
Actualizando a pagina de mentoria dados colectivos e ind
</commit_message>
<xml_diff>
--- a/Qualidade_Sessoes.xlsx
+++ b/Qualidade_Sessoes.xlsx
@@ -10305,13 +10305,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A10AC6AC-8705-469D-8149-D10956DE0CD5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17C03E81-6C94-48BF-8793-32440DC620D9}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFB6F85F-A402-4B53-830F-A99DEA1544D1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB788E5D-2D79-4363-AF59-D9AE6FBE16C9}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D11353ED-4446-4AB4-9FC4-8DD1687CE22E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73DE38E5-A439-4DFE-870D-009DEC8E8546}"/>
 </file>
</xml_diff>